<commit_message>
Refresh the 7/28 report with settled ad spend and the corrected creative calls
Meta's account-level figure for 7/27 settled at 563,415 against the 562,908
summed from campaigns overnight; the report now uses the settled value.

The 7/29 call on the portable shaver is withdrawn. It was declared as cut to
8,000 if 7-day MER stayed under 1.90, but the diagnosis came back as creative
fatigue at -22.9% CTR with frequency flat, and cutting is only right for
demand decay. Both it and the arm cover get a creative added at held budget
with judgment on 8/5.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017JNTxDUfjQsrckfss7YKHj
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-28.xlsx
+++ b/data/reports/report-2026-07-28.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -602,14 +602,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LOOTY ネクストアクション 2026-07-28(火) 定例（昨日=7/27 月実績）</t>
+          <t>LOOTY ネクストアクション 2026-07-28(火) 定例（昨日=7/27 月実績・広告費は確定値に更新）</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>■ 今日やること（広告）— 4件・15分</t>
+          <t>■ 今日やること（広告）</t>
         </is>
       </c>
       <c r="B3" s="3" t="n"/>
@@ -641,7 +641,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>所要</t>
+          <t>状態</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>2分</t>
+          <t>✅ 実施済</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>2分</t>
+          <t>✅ 実施済</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>2分</t>
+          <t>✅ 実施済</t>
         </is>
       </c>
     </row>
@@ -749,335 +749,347 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>2分</t>
+          <t>✅ 実施済</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>接触冷感UVアームカバー にCRを1本追加</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>17,000（据置）</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>CTR 2.52%→2.13%（−15.5%）＝素材疲弊。頻度1.29で擦り切れではない。配信CR1本</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>⏳ 未実施</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>携帯電動シェーバー にCRを1本追加</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>11,000（据置）</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>CTR 3.54%→2.73%（−22.9%）＝口座内で最悪の劣化。配信CR1本。素材がなければ複製リセットで可</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>⏳ 未実施</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>UVハット 新規出稿</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0→13,000</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>①〜③で浮いた23,000円から充当。CJのサイズ・色在庫を確認してから</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>⏳ 未実施</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>■ 今日やること（新規出稿）</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>商品</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>日予算</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>出どころ</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>CR</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>判定</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>完全遮光・接触冷感UVハット</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>13,000</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>①②③で浮く23,000円から充当（差引 全体−10,000円）</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>新規CR＋可能なら予備1本。日傘/パーカーで勝っているオーディエンス設定をコピー</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>8/4: 7日CPA&lt;2,476→増額／&lt;4,569→据置／以上→停止</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>■ 今週の1件（広告以外）</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>商品</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>作業</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>所要</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>期限</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>期待効果</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>判定</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>卓上冷感クーラー</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>カラー/タイプのバリエーション追加（現在Default Title 1種のみ）</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>30分</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>7/31</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>CVR 1.93%(17位/19)→2.5%で +約170,000円/週。残シーズン5週</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>8/3 CVR≥2.5%</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>（実施済）卓上</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>FVに「水を入れる家電」の不安解消ブロックを追加</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>7/27完了</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>8/3</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>（実施済）ムダ毛</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>価格 5,980→6,980円</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>7/27完了</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>+26,181〜45,000円/週</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>8/3 7日販売数≥35個</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>■ 予算の増減サマリー</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr"/>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr"/>
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>変更前</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>変更後</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>差</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>4WAY</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>95,000</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>85,000</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>−10,000</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>完全遮光・UV日傘</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>41,000</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>34,000</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>−7,000</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>接触冷感UVパーカー</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>34,000</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>28,000</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>−6,000</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr"/>
+      <c r="E24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>5WAY腰掛けファン</t>
+          <t>4WAY</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>95,000</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>16,250</t>
+          <t>85,000</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>+3,250</t>
+          <t>−10,000</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr"/>
@@ -1085,22 +1097,22 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>UVハット（新規）</t>
+          <t>完全遮光・UV日傘</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>41,000</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>34,000</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>+13,000</t>
+          <t>−7,000</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr"/>
@@ -1108,129 +1120,129 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
+          <t>接触冷感UVパーカー</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>34,000</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>28,000</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>−6,000</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>5WAY腰掛けファン</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>13,000</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>16,250</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>+3,250</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>UVハット（新規）</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>13,000</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>+13,000</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>582,000</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>575,250</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>−6,750</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>■ 次の判定日（基準は本日宣言。当日は当てはめるだけ）</t>
         </is>
       </c>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="B32" s="3" t="n"/>
+      <c r="C32" s="3" t="n"/>
+      <c r="D32" s="3" t="n"/>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>日付</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>商品</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>合格基準</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>不合格時</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>7/29</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>3WAYサーキュレーター</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>増分MER −3.37 は分岐1.71を割っている → 16,000→13,000に戻す</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>（実施）</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>7/29</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>偏光・調光サングラス</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>余裕 &gt; 0（現+0.54）。D5需要減衰でCPA+21%</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>余裕割れなら段階減額</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>7/29</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>接触冷感UVアームカバー</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>余裕 &gt; 0（現+0.69）。D1素材疲弊 CTR−15%</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>CR追加（予算据置）</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -1240,17 +1252,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>携帯電動シェーバー</t>
+          <t>3WAYサーキュレーター</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>7日MER ≥ 1.90（現1.68・余裕+0.17）</t>
+          <t>増分MER −3.37 は分岐1.71を割っている → 16,000→13,000に戻す</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>11,000→8,000</t>
+          <t>（実施）</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr"/>
@@ -1263,17 +1275,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>バランスケアスリッパ</t>
+          <t>偏光・調光サングラス</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>余裕 &gt; 0（現+1.14）</t>
+          <t>余裕 &gt; 0（現+0.54）。D5需要減衰でCPA+21%</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>据置</t>
+          <t>余裕割れなら段階減額</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr"/>
@@ -1281,22 +1293,22 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>7/30</t>
+          <t>8/5</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>害虫ブロッカー</t>
+          <t>携帯電動シェーバー</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>7/26増額分の増分MER ≥ 分岐1.28</t>
+          <t>【訂正】診断が素材疲弊なので減額しない。CR追加＋予算据置で7日後に 7日MER ≥ 1.90</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>85,000→73,000</t>
+          <t>未達なら11,000→8,000</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr"/>
@@ -1304,22 +1316,22 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>7/30</t>
+          <t>8/5</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>ナノガラス脱毛パッド</t>
+          <t>接触冷感UVアームカバー</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>7/26増額分の増分MER ≥ 分岐1.23</t>
+          <t>【訂正】同上。CR追加＋予算据置で7日後に 余裕 ≥ +0.8</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>68,000→60,000</t>
+          <t>未達なら17,000→13,000</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr"/>
@@ -1327,22 +1339,22 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>7/30</t>
+          <t>7/29</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>UV歯ブラシ除菌器</t>
+          <t>バランスケアスリッパ</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>A-コピーのCPA &lt; 5,000</t>
+          <t>余裕 &gt; 0（現+1.14）</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>減額</t>
+          <t>据置</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr"/>
@@ -1350,22 +1362,22 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>7/31</t>
+          <t>7/30</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>卓上冷感クーラー</t>
+          <t>害虫ブロッカー</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>30,000に戻した後の7日MERが目標3.16以上</t>
+          <t>7/26増額分の増分MER ≥ 分岐1.28</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>再検討</t>
+          <t>85,000→73,000</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr"/>
@@ -1373,22 +1385,22 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>7/31</t>
+          <t>7/30</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>5WAY腰掛けファン</t>
+          <t>ナノガラス脱毛パッド</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>本日の増額分の増分MER ≥ 分岐1.59</t>
+          <t>7/26増額分の増分MER ≥ 分岐1.23</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>16,250→13,000に戻す</t>
+          <t>68,000→60,000</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr"/>
@@ -1396,22 +1408,22 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>7/31</t>
+          <t>7/30</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>秋物の選定（シーズン到来3〜4週前）</t>
+          <t>UV歯ブラシ除菌器</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>A-コピーのCPA &lt; 5,000</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>減額</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr"/>
@@ -1419,22 +1431,22 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>8/1</t>
+          <t>7/31</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>手数料の月次再計測・瞬間冷感ポンチョ・壁掛けディスペンサー</t>
+          <t>卓上冷感クーラー</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>30,000に戻した後の7日MERが目標3.16以上</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>再検討</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr"/>
@@ -1442,22 +1454,22 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>8/3</t>
+          <t>7/31</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>卓上(LP)・害虫(CR)・ムダ毛(値上げ) の効果判定</t>
+          <t>5WAY腰掛けファン</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>各上記</t>
+          <t>本日の増額分の増分MER ≥ 分岐1.59</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>16,250→13,000に戻す</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr"/>
@@ -1465,59 +1477,128 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
+          <t>7/31</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>秋物の選定（シーズン到来3〜4週前）</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>8/1</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>手数料の月次再計測・瞬間冷感ポンチョ・壁掛けディスペンサー</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>8/3</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>卓上(LP)・害虫(CR)・ムダ毛(値上げ) の効果判定</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>各上記</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
           <t>8/4</t>
         </is>
       </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>完全遮光・接触冷感UVハット</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr">
         <is>
           <t>7日CPA &lt; 2,476円</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>4,569円以上なら停止</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="E47" s="5" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>■ フローの修正（本日発覚）</t>
         </is>
       </c>
-      <c r="B46" s="3" t="n"/>
-      <c r="C46" s="3" t="n"/>
-      <c r="D46" s="3" t="n"/>
-      <c r="E46" s="3" t="n"/>
-      <c r="F46" s="3" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="B49" s="3" t="n"/>
+      <c r="C49" s="3" t="n"/>
+      <c r="D49" s="3" t="n"/>
+      <c r="E49" s="3" t="n"/>
+      <c r="F49" s="3" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>S1b を追加。平均MERが目標未達の商品は S2→S2a へ逸れて S5 の増分判定に到達せず、宣言した「増分MER&lt;分岐なら戻す」が実行されなかった。完全遮光とパーカーがこれに該当し、本来の減額が出ていなかった。</t>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr"/>
-      <c r="C47" s="4" t="inlineStr"/>
-      <c r="D47" s="4" t="inlineStr"/>
-      <c r="E47" s="4" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr"/>
+      <c r="C50" s="4" t="inlineStr"/>
+      <c r="D50" s="4" t="inlineStr"/>
+      <c r="E50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>修正後: 7日利益が黒字なら、平均MERの水準に関係なく、まず「直近の増額分の増分MERが分岐を割っていないか」を見る。割っていれば元の予算に戻す（外せば必ず利益が増えるため）。</t>
         </is>
       </c>
-      <c r="B48" s="5" t="inlineStr"/>
-      <c r="C48" s="5" t="inlineStr"/>
-      <c r="D48" s="5" t="inlineStr"/>
-      <c r="E48" s="5" t="inlineStr"/>
+      <c r="B51" s="5" t="inlineStr"/>
+      <c r="C51" s="5" t="inlineStr"/>
+      <c r="D51" s="5" t="inlineStr"/>
+      <c r="E51" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1530,7 +1611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1547,7 +1628,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>LOOTY 日次損益レポート 2026-07-28(火) 定例（昨日=7/27 月実績）</t>
+          <t>LOOTY 日次損益レポート 2026-07-28(火) 定例（昨日=7/27 月実績・広告費は確定値に更新）</t>
         </is>
       </c>
     </row>
@@ -1654,21 +1735,21 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>562908</v>
+        <v>563415</v>
       </c>
       <c r="C7" s="8" t="inlineStr"/>
       <c r="D7" s="9" t="n">
-        <v>581833</v>
+        <v>582042</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>559009</v>
+        <v>559098</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>476437</v>
+        <v>476458</v>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>+0.7%</t>
+          <t>+0.8%</t>
         </is>
       </c>
     </row>
@@ -1679,21 +1760,21 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>263017</v>
+        <v>262510</v>
       </c>
       <c r="C8" s="8" t="inlineStr"/>
       <c r="D8" s="9" t="n">
-        <v>397215</v>
+        <v>397005</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>442194</v>
+        <v>442105</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>442290</v>
+        <v>442269</v>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>-40.5%</t>
+          <t>-40.6%</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1807,7 @@
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>-8.5pt</t>
+          <t>-8.6pt</t>
         </is>
       </c>
     </row>
@@ -1737,21 +1818,21 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>221932</v>
+        <v>221425</v>
       </c>
       <c r="C10" s="8" t="inlineStr"/>
       <c r="D10" s="9" t="n">
-        <v>348573</v>
+        <v>348363</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>392192</v>
+        <v>392103</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>397031</v>
+        <v>397010</v>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>-43.4%</t>
+          <t>-43.5%</t>
         </is>
       </c>
     </row>
@@ -1822,22 +1903,22 @@
         <v>351303</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>562908</v>
+        <v>563415</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>263017</v>
+        <v>262510</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>0.2234</v>
+        <v>0.223</v>
       </c>
       <c r="G14" s="10" t="n">
         <v>41085</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>221932</v>
+        <v>221425</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.1885</v>
+        <v>0.1881</v>
       </c>
     </row>
     <row r="15">
@@ -1853,22 +1934,22 @@
         <v>1244114</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>1745498</v>
+        <v>1746126</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>1191644</v>
+        <v>1191016</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>0.285</v>
+        <v>0.2848</v>
       </c>
       <c r="G15" s="10" t="n">
         <v>145926</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>1045718</v>
+        <v>1045090</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.2501</v>
+        <v>0.2499</v>
       </c>
     </row>
     <row r="16">
@@ -1884,10 +1965,10 @@
         <v>3020633</v>
       </c>
       <c r="D16" s="10" t="n">
-        <v>3913060</v>
+        <v>3913688</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>3095361</v>
+        <v>3094733</v>
       </c>
       <c r="F16" s="11" t="n">
         <v>0.3086</v>
@@ -1896,7 +1977,7 @@
         <v>350014</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>2745347</v>
+        <v>2744719</v>
       </c>
       <c r="I16" s="11" t="n">
         <v>0.2737</v>
@@ -1915,22 +1996,22 @@
         <v>11343303</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>14293116</v>
+        <v>14293744</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>13268707</v>
+        <v>13268079</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>0.3411</v>
+        <v>0.341</v>
       </c>
       <c r="G17" s="10" t="n">
         <v>1357789</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>11910918</v>
+        <v>11910290</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>0.3062</v>
+        <v>0.3061</v>
       </c>
     </row>
     <row r="18">
@@ -1946,10 +2027,10 @@
         <v>4277098</v>
       </c>
       <c r="D18" s="10" t="n">
-        <v>5511288</v>
+        <v>5511916</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>4430786</v>
+        <v>4430158</v>
       </c>
       <c r="F18" s="11" t="n">
         <v>0.3116</v>
@@ -1958,7 +2039,7 @@
         <v>496249</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>3934537</v>
+        <v>3933909</v>
       </c>
       <c r="I18" s="11" t="n">
         <v>0.2767</v>
@@ -1974,75 +2055,89 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>・★本日の判定4件はすべて7/27までに宣言済みの基準に機械的に当てはめた結果。新しい理由づけは加えていない</t>
+          <t>・★本日の判定4件はすべて7/27までに宣言済みの基準に機械的に当てはめた結果。新しい理由づけは加えていない。4件とも実施済み</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>・★増額分の巻き戻し3件で合計23,000円/日を回収。うち13,000円をUVハットの新規出稿へ、3,250円を5WAYの増額へ再配分し、差引で全体−6,750円/日</t>
+          <t>・★訂正: 携帯電動シェーバーの7/29判定を「7日MER&lt;1.90なら減額」と宣言していたが、診断が D1素材疲弊（CTR −22.9%）と出たため取り下げる。減額が正解なのは D5需要減衰 と診断されたときだけ。素材疲弊は CR追加＋予算据置＋7日後判定（8/5）が正しい。接触冷感UVアームカバー（CTR −15.5%）も同じ扱いにする</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>・★増分MERは「直近の1段」を測る。P1・P2とも予算変更日をまたがず、①曜日指数補正と②全店コントロール補正の2通りで算出し、両方が同じゾーン（&lt;分岐／分岐〜目標／≥目標）に落ちたときだけ採用する</t>
+          <t>・★CR投入トリガーを全18商品で点検した結果、必要なのは 接触冷感UVアームカバー と 携帯電動シェーバー の2つだけ。バランスケアスリッパは7/23の半減後にCTR+8.5%・CPA−6.3%・CVR自店4位と全指標が改善しており、CR3本もすでに入っているため不要</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>・★CVRは自店19商品の順位で評価する（中央値 3.19%）。前週比だけでLP改善と判断しない。下位25%＝ディスペンサー1.60%(19位)・ワンピース1.84%(18位)・卓上1.93%(17位)・3WAY2.66%(16位)・UV歯ブラシ2.85%(15位)</t>
+          <t>・★増額分の巻き戻し3件で合計23,000円/日を回収。うち13,000円をUVハットの新規出稿へ、3,250円を5WAYの増額へ再配分し、差引で全体−6,750円/日</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>・★残シーズン週数を打ち手の選定に使う。残5週未満（卓上・4WAY・5WAY・3WAY）には原価交渉を提案しない（反映まで3〜4週かかり回収できない）</t>
+          <t>・★増分MERは「直近の1段」を測る。P1・P2とも予算変更日をまたがず、①曜日指数補正と②全店コントロール補正の2通りで算出し、両方が同じゾーン（&lt;分岐／分岐〜目標／≥目標）に落ちたときだけ採用する</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>・曜日指数(30日実測): 日117・水105・土102・金99・月95・木93・火86</t>
+          <t>・★CVRは自店19商品の順位で評価する（中央値 3.19%）。前週比だけでLP改善と判断しない。下位25%＝ディスペンサー1.60%(19位)・ワンピース1.84%(18位)・卓上1.93%(17位)・3WAY2.66%(16位)・UV歯ブラシ2.85%(15位)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>・★増額候補（自分の目標MER超え × 消化率95%以上）: 4WAY 取り付けOK (3.37&gt;3.30・103%)・形状記憶日傘(3.52&gt;2.58・99%)・害虫ブロッカー(2.66&gt;2.31・100%)・ナノガラス脱毛パッド(2.47&gt;2.17・96%)・卓上冷感クーラー(3.43&gt;3.16・102%)・5WAY腰掛けファン(4.11&gt;3.59・100%)・瞬間冷感ポンチョ(2.71&gt;2.49・100%)</t>
+          <t>・★残シーズン週数を打ち手の選定に使う。残5週未満（卓上・4WAY・5WAY・3WAY）には原価交渉を提案しない（反映まで3〜4週かかり回収できない）</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>・全期間の売上・原価・広告費はShopify/Metaの実測。推計・外挿・平均の流用は不使用。ナノガラス脱毛パッド・壁掛けディスペンサーはバリエーション別の実販売数で原価を加重（30日も実測）</t>
+          <t>・曜日指数(30日実測): 日117・水105・土102・金99・月95・木93・火86</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>・累積行は日次実測から毎回積み直し、構成日の合計と一致することをコード内でassertしている（繰り越し加算は使わない）</t>
+          <t>・★増額候補（自分の目標MER超え × 消化率95%以上）: 4WAY 取り付けOK (3.37&gt;3.30・103%)・形状記憶日傘(3.52&gt;2.58・99%)・害虫ブロッカー(2.66&gt;2.31・100%)・ナノガラス脱毛パッド(2.47&gt;2.17・96%)・卓上冷感クーラー(3.43&gt;3.16・102%)・5WAY腰掛けファン(4.11&gt;3.59・100%)・瞬間冷感ポンチョ(2.71&gt;2.49・100%)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>・30日窓の途中開始: 卓上冷感クーラー7/13(15日)・5WAY腰掛けファン7/19(9日)・瞬間冷感ポンチョ/ムダ毛シェーバー7/10(18日)</t>
+          <t>・全期間の売上・原価・広告費はShopify/Metaの実測。推計・外挿・平均の流用は不使用。ナノガラス脱毛パッド・壁掛けディスペンサーはバリエーション別の実販売数で原価を加重（30日も実測）</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>・累積行は日次実測から毎回積み直し、構成日の合計と一致することをコード内でassertしている（繰り越し加算は使わない）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>・30日窓の途中開始: 卓上冷感クーラー7/13(15日)・5WAY腰掛けファン7/19(9日)・瞬間冷感ポンチョ/ムダ毛シェーバー7/10(18日)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>・害虫ブロッカー本体(70,000円)は7/27にCRが1本→3本に増えた（A / B-コピー / A-コピー）。効果判定は8/3</t>
         </is>
@@ -4375,7 +4470,7 @@
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>姿勢サポートベルト</t>
+          <t>ナノバブルシャワーヘッド</t>
         </is>
       </c>
       <c r="B24" s="10" t="n">
@@ -4420,7 +4515,7 @@
       </c>
       <c r="R24" s="8" t="inlineStr"/>
       <c r="S24" s="10" t="n">
-        <v>4551</v>
+        <v>37800</v>
       </c>
       <c r="T24" s="8" t="inlineStr"/>
       <c r="U24" s="8" t="inlineStr"/>
@@ -4449,7 +4544,7 @@
     <row r="25">
       <c r="A25" s="20" t="inlineStr">
         <is>
-          <t>ナノバブルシャワーヘッド</t>
+          <t>リカバリーサンダル</t>
         </is>
       </c>
       <c r="B25" s="21" t="n">
@@ -4494,7 +4589,7 @@
       </c>
       <c r="R25" s="20" t="inlineStr"/>
       <c r="S25" s="21" t="n">
-        <v>37800</v>
+        <v>18697</v>
       </c>
       <c r="T25" s="20" t="inlineStr"/>
       <c r="U25" s="20" t="inlineStr"/>
@@ -4523,7 +4618,7 @@
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>ネックマッサージャー</t>
+          <t>姿勢サポートベルト</t>
         </is>
       </c>
       <c r="B26" s="10" t="n">
@@ -4568,7 +4663,7 @@
       </c>
       <c r="R26" s="8" t="inlineStr"/>
       <c r="S26" s="10" t="n">
-        <v>6946</v>
+        <v>4551</v>
       </c>
       <c r="T26" s="8" t="inlineStr"/>
       <c r="U26" s="8" t="inlineStr"/>
@@ -4597,7 +4692,7 @@
     <row r="27">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>リカバリーサンダル</t>
+          <t>ネックマッサージャー</t>
         </is>
       </c>
       <c r="B27" s="21" t="n">
@@ -4642,7 +4737,7 @@
       </c>
       <c r="R27" s="20" t="inlineStr"/>
       <c r="S27" s="21" t="n">
-        <v>18697</v>
+        <v>6946</v>
       </c>
       <c r="T27" s="20" t="inlineStr"/>
       <c r="U27" s="20" t="inlineStr"/>

</xml_diff>

<commit_message>
Reissue the 7/28 report on the unchanged product-sales definition
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017JNTxDUfjQsrckfss7YKHj
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-28.xlsx
+++ b/data/reports/report-2026-07-28.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -602,14 +602,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LOOTY ネクストアクション 2026-07-28(火) 定例（昨日=7/27 月実績）【監査確定版・基準は手数料控除前で統一】</t>
+          <t>LOOTY ネクストアクション 2026-07-28(火) 定例（昨日=7/27 月実績）</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>■ 🚨 監査による訂正（本日中に実施）</t>
+          <t>■ 今日やること（4件・20分）</t>
         </is>
       </c>
       <c r="B3" s="3" t="n"/>
@@ -631,15 +631,19 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>現→修正</t>
+          <t>現→変更</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>理由</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr"/>
+          <t>根拠</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>状態</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -649,7 +653,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>接触冷感UVパーカーの予算を戻す</t>
+          <t>接触冷感UVパーカー の予算を戻す</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -659,12 +663,12 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>今朝の減額は増分MERの計測バグ（P1の7/20広告費欠落）による誤指示。修正後の実測は曜日+2.36/全店+5.35で、増額分は実効分岐1.78を超えて黒字だった</t>
+          <t>今朝の減額は増分MERの計測ミス（P1の7/20広告費がデータ欠落しゼロ扱い）による誤指示。修正後の実測は曜日+2.36 / 全店+5.35で、いずれも分岐1.56を超え＝増額分は黒字だった</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>⏳</t>
+          <t>⏳ 未実施</t>
         </is>
       </c>
     </row>
@@ -676,266 +680,314 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>【撤回】7/29の3WAY巻き戻し(16,000→13,000)は行わない</t>
+          <t>接触冷感UVアームカバー にCRを1本追加</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>16,000 据置</t>
+          <t>17,000（据置）</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Δ広告費の実測が2,163円/日&lt;3,000で測定不能（V1）。−3.37という値も同じデータ欠落の産物</t>
+          <t>CTR 2.52%→2.13%（−15.5%）＝素材疲弊。頻度1.29で擦り切れではなく純粋な素材劣化。配信CR1本</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⏳ 未実施</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>携帯電動シェーバー にCRを1本追加</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>11,000（据置）</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>CTR 3.54%→2.73%（−22.9%）＝口座内で最悪の劣化。余裕+0.17と全商品で最小のため優先度高。減額ではなくCR追加が正解（診断が素材疲弊のため）</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>⏳ 未実施</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>■ 実施済み（監査で再検証OK）</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>完全遮光・接触冷感UVハット 新規出稿</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0→13,000</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>原価率23.6%・目標MER2.42。日傘/パーカーで勝っているオーディエンス設定をコピー。CJのサイズ・色在庫を確認してから</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>⏳ 未実施</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>■ 実施済み（本日の予算判定4件・すべて宣言済み基準どおり）</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>操作</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>増分MER（修正後の確定値）</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>増分MER（データ修正後の確定値）</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>分岐</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>判定</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>卓上 38,000→30,000</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>曜日−9.55 / 全店−9.49</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>✅ 正しい</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>4WAY 95,000→85,000</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>曜日−8.73 / 全店−8.41</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>✅ 正しい</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>完全遮光 41,000→34,000</t>
+          <t>4WAY 95,000→85,000</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>曜日−7.99 / 全店−5.17</t>
+          <t>曜日−8.73 / 全店−8.41</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
           <t>✅ 正しい</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>5WAY 13,000→16,250</t>
+          <t>完全遮光 41,000→34,000</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>未測定→+25%プローブ</t>
+          <t>曜日−7.99 / 全店−5.17</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>✅ フロー通り（7/31判定の合格線は実効分岐1.81に更新）</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr"/>
+          <t>1.35</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>✅ 正しい</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>ディスペンサー 6,000維持</t>
+          <t>卓上 38,000→30,000（7/27実施）</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>削った分は+1.3〜1.5&lt;実効分岐1.49</t>
+          <t>曜日−9.55 / 全店−9.49</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>✅ 減額は正解・維持（方向対応S1bで確認）</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>■ 残タスク</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>✅ 正しい</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>5WAY 13,000→16,250</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>未測定→+25%で測定可能にする</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>1.59</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>✅ フロー通り（7/31判定）</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>操作</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>内容</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>■ 取り消した指示（監査で判明）</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>アームカバーにCR1本</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>17,000円据置。CTR−15.5%＝素材疲弊。8/5判定</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr"/>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>対象</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>当初の指示</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>取り消しの理由</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>携帯シェーバーにCR1本</t>
+          <t>接触冷感UVパーカー</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>11,000円据置。CTR−22.9%。余裕+0.17⚠️（手数料込みでは赤字圏）のため優先。8/5判定 MER≥1.90</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr"/>
+          <t>34,000→28,000に減額</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>増分MERの計測に使うP1期間の広告費データが1日分欠落しゼロ扱いになり、+2.4〜+5.4を+0.93と誤計測していた。修正後は分岐超えで、減額は不要だった</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>UVハット新規出稿 13,000円</t>
+          <t>3WAYサーキュレーター（7/29予定）</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>CJ在庫確認後。停止線は分岐CPA 4,569円</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>■ 更新後の判定カレンダー（しきい値を実効分岐に張り替え）</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
+          <t>16,000→13,000に戻す</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>7/23の変更は実測Δ広告費が2,163円/日で、測定下限3,000円に届かない＝増分MERを算出してはいけない実験だった。16,000円で据置</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>携帯電動シェーバー（7/29予定）</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>7日MER&lt;1.90なら11,000→8,000に減額</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>診断が素材疲弊（CTR−22.9%）。減額が正解なのは需要減衰のときだけ。CR追加＋予算据置に変更し、判定を8/5へ</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>■ 次の判定日（基準は本日宣言・当日は当てはめるだけ）</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>日付</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>商品</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>基準（手数料控除前で統一）</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>合格基準</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>不合格時</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>7/29</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>害虫ブロッカー・ナノガラス</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>【自動導出で7/30→7/29】7/26増額分の増分MER ≥ 分岐（1.28 / 1.23）。害虫はP2に7/27のCR学習が混入するため証拠不足なら8/1へ延期</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>85,000→73,000 / 68,000→60,000</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -945,89 +997,85 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>サングラス</t>
+          <t>害虫ブロッカー</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>余裕+0.54 &gt; 0 → 据置。D5需要減衰は2週連続確認ルールで8/4に再確認</t>
+          <t>7/26増額分（73,000→85,000）の増分MER ≥ 分岐1.28。ただしP2に7/27のCR投入（学習期）が混入するため、証拠不足なら8/1へ延期</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr"/>
+          <t>85,000→73,000</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>7/30</t>
+          <t>7/29</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>UV歯ブラシ</t>
+          <t>ナノガラス脱毛パッド</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>A-コピーのCPA &lt; 5,000（購入10件未満なら延期・V9）</t>
+          <t>7/26増額分（60,000→68,000）の増分MER ≥ 分岐1.23</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>減額</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr"/>
+          <t>68,000→60,000</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>7/31</t>
+          <t>7/29</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>5WAY</t>
+          <t>偏光・調光サングラス</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>増額分の増分MER ≥ 分岐1.59</t>
+          <t>余裕 &gt; 0（現+0.54）。D5需要減衰でCPA+21%</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>16,250→13,000</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr"/>
+          <t>余裕割れなら段階減額</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>7/31</t>
+          <t>7/30</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>巻き戻し4件の回復確認</t>
+          <t>UV歯ブラシ除菌器</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>卓上・4WAY・完全遮光の7日MERが巻き戻し前水準へ回復／パーカー34,000復帰後の実測</t>
+          <t>A-コピーのCPA &lt; 5,000（購入10件未満なら証拠不足で延期）</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr"/>
+          <t>減額</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1037,58 +1085,56 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>秋物選定（シーズン到来3〜4週前）</t>
+          <t>5WAY腰掛けファン</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>本日の増額分の増分MER ≥ 分岐1.59</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr"/>
+          <t>16,250→13,000</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>8/3</t>
+          <t>7/31</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>卓上(LP CVR≥2.5%)・害虫(CR CTR≥3.0%)・ムダ毛(7日販売数≥35個)</t>
+          <t>巻き戻し3件の回復確認</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>効果判定</t>
+          <t>卓上・4WAY・完全遮光の7日MERが巻き戻し前の水準へ戻っているか</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>各基準参照</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>8/4-5</t>
+          <t>7/31</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>UVハット(停止線CPA4,569)・アームカバー(余裕≥+0.8)・携帯シェーバー(MER≥1.90)</t>
+          <t>秋物の選定（シーズン到来3〜4週前）</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>CR/出稿の効果判定</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -1096,73 +1142,174 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>8/1</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>手数料の月次再計測・瞬間冷感ポンチョ・壁掛けディスペンサー</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>■ LP改善対象の訂正（価格帯を無視したCVR順位は誤り）</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="n"/>
-      <c r="C33" s="3" t="n"/>
-      <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="n"/>
-      <c r="F33" s="3" t="n"/>
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>8/3</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>卓上(LP CVR≥2.5%)・害虫(CR CTR≥3.0%)・ムダ毛(7日販売数≥35個)</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>本日までの施策の効果判定</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>各基準参照</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>評価</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>商品</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>売上/クリック（中央値209円）</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr"/>
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>8/4</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>UVハット</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>7日CPA &lt; 2,476円→増額 ／ &lt; 4,569円→据置</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>4,569円以上なら停止</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>🚨 対象</t>
+          <t>8/5</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>ディスペンサー113円・サングラス135円・卓上152円・携帯シェーバー154円</t>
+          <t>アームカバー(余裕≥+0.8)・携帯シェーバー(7日MER≥1.90)</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>同価格帯内でも劣後</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>✅ 取り消し</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>UV歯ブラシ（329円=店内2位）・3WAY（234円）</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>CVR順位が低いのは高単価のせいでLPは健全。昨日のLP改善提案を撤回</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr"/>
+          <t>CR追加の効果判定</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>未達なら減額</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>■ LP改善の対象（価格帯を考慮して再評価）</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="3" t="n"/>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>評価</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>商品</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>売上/クリック（店内中央値209円）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>🚨 改善対象</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>壁掛けディスペンサー113円・偏光サングラス135円・卓上冷感クーラー152円・携帯電動シェーバー154円</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>同価格帯の商品と比べても劣後</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>✅ 対象外に訂正</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>UV歯ブラシ除菌器（329円＝店内2位）・3WAYサーキュレーター（234円）</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>CVR順位が低いのは単価が高いためでLPは健全。前日のLP改善提案を撤回</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>✅ 触らない</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>4WAY・アームカバー・パーカー・害虫・ムダ毛・スリッパほか</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>CVRが自店の中央値以上</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1175,7 +1322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1192,7 +1339,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>LOOTY 日次損益レポート 2026-07-28(火) 定例（昨日=7/27 月実績）【監査確定版・基準は手数料控除前で統一】</t>
+          <t>LOOTY 日次損益レポート 2026-07-28(火) 定例（昨日=7/27 月実績）</t>
         </is>
       </c>
     </row>
@@ -1612,63 +1759,84 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>・【監査 2026-07-28】増分MERの計測にデータ欠落バグ（7日窓のスライドでP1の7/20広告費が0円扱い）。パーカーの巻き戻し(34,000→28,000)は誤指示だったため取り消し。卓上・4WAY・完全遮光の巻き戻しは修正後データでも正しいことを再確認</t>
+          <t>・売上=gross_sales−discounts（返品A案）。商品別の売上はgross、値引は全体サマリーで一括控除（2026-07-20の規約どおり・変更なし）。MER・分岐MER・目標MER・増分MERはすべて手数料控除前で統一</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>・【確定】MER・分岐・目標・増分MERはすべて手数料控除前で統一（2026-07-28ユーザー決定）。実効分岐は判定に使わず、余裕&lt;0.20の商品への⚠️注記のみ（携帯電動シェーバー+0.17⚠️）。手数料控除後の現金は全体サマリーの「控除後利益」行で把握する</t>
+          <t>・★本日の判定4件はすべて7/27までに宣言済みの基準に機械的に当てはめた結果。新しい理由づけは加えていない</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>・【監査】曜日指数から祝日(7/20海の日)を除外。月曜指数94.8→88.2。「7/27は同曜日比−5.0%」は誤りで、実際は非祝日月曜平均比+2.9%＝平常。弱かったのは売上ではなく効率のみ</t>
+          <t>・★【重要な訂正】増分MERの計測に、広告費データの取得窓がスライドしてP1の一部日付が欠落しゼロ扱いになるバグがあった。これにより接触冷感UVパーカーの巻き戻し指示（34,000→28,000）を誤って発行した。再発防止としてP1・P2の全日付が広告費データに存在することを毎回assertする（V5）</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>・【監査】増分MERの負値は「増額分の追加売上が検出されず(≒0以下)」と読む。増額は好調期の直後に行われがちで平均回帰によりP1が上振れ＝負に偏るため、値の絶対値は文字通りに受け取らない</t>
+          <t>・★増分MERは「直近の1段」を測る。P1・P2とも予算変更日をまたがず、祝日を除外し、①曜日指数補正 ②全店コントロール補正 の2通りで算出して、両方が同じゾーンに落ちたときだけ採用する</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>・【監査】週次MER実測: 7/07-13 2.66 → 7/14-20 2.68 → 7/21-27 2.56。効率は横ばいではなく直近週で−4%＝夏物ピークアウトの初期シグナル。日傘ペアは全店−9.6%に対し−20.7%と先行して減衰（完全遮光の巻き戻しと整合）</t>
+          <t>・★曜日指数から祝日（7/20 海の日）を除外。月曜指数 94.8→88.2。7/27は「同曜日比−5.0%」ではなく非祝日月曜平均比+2.9%＝売上は平常。弱かったのは効率のみ</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>・【監査】測定ガードV5〜V9を追加: データ被覆assert・祝日除外・負値の解釈・コントロール汚染除去・最小25購入。判定フローS1bは方向対応に修正（減額実験に対して逆作動するバグを未然に修正）</t>
+          <t>・★増分MERの負値は「増額分の追加売上が検出されなかった（実質ゼロ以下）」と読む。広告が売上を消すことはなく、増額は好調期の直後に行われがちで平均回帰により負に偏るため。分岐割れという結論自体は頑健</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>・売上=gross_sales−discounts（返品A案）。当月返品累計 7/27時点 197,584円（返品率0.55%）</t>
+          <t>・★週次MER（完結週・全店実測）: 7/07-13 2.66 → 7/14-20 2.68 → 7/21-27 2.56。直近週で−4%＝夏物ピークアウトの初期シグナル。日傘ペアは全店−9.6%に対し−20.7%と先行して減衰。8月上旬は増額より秋物テストの準備へ</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>・全期間の売上・原価・広告費はShopify/Metaの実測。累積行は日次から毎回積み直し</t>
+          <t>・★収益算定の照合（毎回assert）: ①Σ商品gross = 全店gross（差0円）②Σ商品利益 − 全店値引 − カタログ広告費 = 全店利益（差+507円=0.02%。Meta当日値の確定ドリフト分）③Σキャンペーン広告費 ≒ アカウントレベル（前日分は翌朝に再取得して確定値に更新）</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>・【v2.0】判定日・実験定義は scripts/experiments.py が budget-snapshots.csv の差分から自動導出（手書き禁止）。天候: 冷感カテゴリの売上シェアが8日で27〜44%と変動＝外部要因実在。気温モデルは作らず、同カテゴリコントロール・極端日の除外・D5の2週確認で測定を保護する</t>
+          <t>・★既知のバイアス（開示のみ・数値は直さない）: 売上はgross（返品を引かない）だが数量は返品分を引くため、返品された数量の原価が原価から消え利益が過大になる。実測 約73,000円/30日（2,440円/日）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>・★値引の正体はクーポンではなく自動割引「Quantity break（2個以上で10%OFF）」。まとめ買いされる商品ほど値引率が高い（7日実測: 害虫9.2%・ポンチョ7.1%・5WAY6.4% ↔ ムダ毛0.5%・携帯0%）。商品別売上はgrossのままなので、これらの商品のMERは実額よりその率だけ良く見える点を判定時に割り引いて読む</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>・全期間の売上・原価・広告費はShopify/Metaの実測。累積行は日次実測から毎回積み直し、構成日の合計と一致することをassert</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>・当月返品累計 7/27時点 197,584円（返品率0.55%）。7/27の新規返品ゼロ</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2628,7 @@
       </c>
       <c r="AD7" s="24" t="inlineStr">
         <is>
-          <t>【広告】41,000→34,000円/日 ／ 【診断】D5需要減衰（CTR/CVR/CPM横ばいでCPAのみ +16%） ／ 【LP】CVR 2.94%＝自店13位/19（中央値以上→LPは触らない） ／ 【広告費率】40%超（率のために黒字は削らない） ／ 【増分MER実測】曜日−7.99 / 全店−5.17（祝日除外・データ補完後の確定値）（曜日・全店の2手法が一致→採用）</t>
+          <t>【広告】41,000→34,000円/日 ／ 【診断】D5需要減衰（CTR/CVR/CPM横ばいでCPAのみ +16%） ／ 【LP】CVR 2.94%＝自店13位/19（中央値以上→LPは触らない） ／ 【広告費率】40%超（率のために黒字は削らない） ／ 【増分MER実測】曜日−7.99 / 全店−5.17（曜日・全店の2手法が一致→採用）</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3610,7 @@
       </c>
       <c r="AD17" s="24" t="inlineStr">
         <is>
-          <t>【実効赤字】表示は7日+8,752円だが値引4.4%+手数料3.49%を配賦すると−1,234円（MER1.68&lt;実効分岐1.71） ／ 【広告】据置（次回判定 7/29） ／ 【診断】D1素材疲弊（CTR 3.54%→2.73% (-23%)） ／ 【LP】CVR 3.20%＝自店8位/19（中央値以上→LPは触らない） ／ 【原価】原価率33.7%&gt;33%。通年なのでCJ数量交渉が有効／+1,000円で数量−23.6%まで許容 ／ 【広告費率】40%超（率のために黒字は削らない）</t>
+          <t>【注意】余裕+0.17は全商品で最小。分岐1.51まであとわずか ／ 【広告】据置（次回判定 7/29） ／ 【診断】D1素材疲弊（CTR 3.54%→2.73% (-23%)） ／ 【LP】CVR 3.20%＝自店8位/19（中央値以上→LPは触らない） ／ 【原価】原価率33.7%&gt;33%。通年なのでCJ数量交渉が有効／+1,000円で数量−23.6%まで許容 ／ 【広告費率】40%超（率のために黒字は削らない）</t>
         </is>
       </c>
     </row>

</xml_diff>